<commit_message>
README con el isotipo, la apertura y el recorrido animados; manuales, notas técnicas y decisiones de la versión 3
- README en español e inglés: isotipo de VicMar, sección de identidad visual, GIF de la apertura y del recorrido, capturas nuevas.
- Manual de usuario reescrito para los tres roles y las pantallas actuales; manuales regenerados en Word.
- ADR-005 y DT-05 con la comparación real de los cuatro modelos (LightGBM elegido por validación cruzada).
- Verificador de coherencia del Avance 2 apuntando a los artefactos actuales.
- Retiro de archivos y referencias del enfoque anterior.
</commit_message>
<xml_diff>
--- a/documentacion/decisiones/Matriz_decisiones.xlsx
+++ b/documentacion/decisiones/Matriz_decisiones.xlsx
@@ -61,7 +61,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -69,6 +69,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -628,19 +629,19 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>LightGBM ajustado con Optuna</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.9</v>
+        <v>4.65</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Gradient boosting (HistGradientBoosting)</t>
+          <t>Random Forest con pesos por clase</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>4.25</v>
+        <v>4.3</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -1366,188 +1367,229 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Criterio (peso)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Random Forest</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Gradient boosting (HistGradientBoosting)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>LightGBM ajustado con Optuna</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Random Forest con pesos por clase</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Regresión logística</t>
         </is>
       </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Random Forest con SMOTE</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Discriminación en datos reales (ROC-AUC en OULAD) (35 %)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Detección de la clase minoritaria (PR-AUC en OULAD) (15 %)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Desempeño en la segunda institución (ROC-AUC en UNEMI_PRUEBAS) (10 %)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Explicación por alumno (15 %)</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Explicación por estudiante (15 %)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Evidencia en trabajos previos (15 %)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Costo de entrenamiento (10 %)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Puntaje ponderado (sobre 5)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>4,90</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>4,25</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>3,85</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>4,65</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>4,30</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>3,75</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>2,70</t>
         </is>
       </c>
     </row>

</xml_diff>